<commit_message>
Adding start and end timestamps to docs from person-create
</commit_message>
<xml_diff>
--- a/forms/contact/person-create.xlsx
+++ b/forms/contact/person-create.xlsx
@@ -4,7 +4,7 @@
   <fileVersion lastEdited="4" lowestEdited="4" rupBuild="3820"/>
   <workbookPr date1904="0"/>
   <bookViews>
-    <workbookView activeTab="2" windowWidth="19200" windowHeight="6620"/>
+    <workbookView activeTab="0" windowWidth="19200" windowHeight="6620"/>
   </bookViews>
   <sheets>
     <sheet name="survey" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="23" count="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="24" count="24">
   <si>
     <t>type</t>
   </si>
@@ -90,10 +90,13 @@
     <t>meta</t>
   </si>
   <si>
+    <t>start</t>
+  </si>
+  <si>
+    <t>end</t>
+  </si>
+  <si>
     <t>yes_no</t>
-  </si>
-  <si>
-    <t>form_title</t>
   </si>
 </sst>
 </file>
@@ -186,7 +189,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:Q49"/>
+  <dimension ref="A1:Q51"/>
   <sheetFormatPr defaultRowHeight="13"/>
   <cols>
     <col min="1" max="1" style="0" width="26.863281249999996" bestFit="1" customWidth="1"/>
@@ -1014,32 +1017,18 @@
     </row>
     <row r="41" spans="1:17" ht="13.5">
       <c r="A41" t="s">
-        <v>11</v>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>created_by</t>
-        </is>
-      </c>
-      <c r="L41" t="inlineStr">
-        <is>
-          <t>../../../name</t>
-        </is>
+        <v>21</v>
+      </c>
+      <c r="B41" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="42" spans="1:17" ht="13.5">
       <c r="A42" t="s">
-        <v>11</v>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>created_by_person_uuid</t>
-        </is>
-      </c>
-      <c r="L42" t="inlineStr">
-        <is>
-          <t>../../../contact_id</t>
-        </is>
+        <v>22</v>
+      </c>
+      <c r="B42" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="43" spans="1:17" ht="13.5">
@@ -1048,36 +1037,66 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>created_by_place_uuid</t>
+          <t>created_by</t>
         </is>
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>../../../facility_id</t>
+          <t>../../../name</t>
         </is>
       </c>
     </row>
     <row r="44" spans="1:17" ht="13.5">
       <c r="A44" t="s">
-        <v>10</v>
-      </c>
-      <c r="B44" t="s">
-        <v>20</v>
+        <v>11</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>created_by_person_uuid</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>../../../contact_id</t>
+        </is>
       </c>
     </row>
     <row r="45" spans="1:17" ht="13.5">
       <c r="A45" t="s">
+        <v>11</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>created_by_place_uuid</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>../../../facility_id</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" spans="1:17" ht="13.5">
+      <c r="A46" t="s">
         <v>10</v>
       </c>
-      <c r="B45" t="s">
+      <c r="B46" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="47" spans="1:17" ht="13.5">
+      <c r="A47" t="s">
+        <v>10</v>
+      </c>
+      <c r="B47" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="47" spans="1:17">
-      <c r="D47" s="1"/>
     </row>
     <row r="49" spans="1:17">
       <c r="D49" s="1"/>
+    </row>
+    <row r="51" spans="1:17">
+      <c r="D51" s="1"/>
     </row>
   </sheetData>
   <sheetProtection formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" selectLockedCells="1" sort="0" autoFilter="0" pivotTables="0" selectUnlockedCells="1"/>
@@ -1124,7 +1143,7 @@
     </row>
     <row r="2" spans="1:4" ht="14.75">
       <c r="A2" s="3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>16</v>
@@ -1142,7 +1161,7 @@
     </row>
     <row r="3" spans="1:4" ht="14.75">
       <c r="A3" s="3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
@@ -1230,8 +1249,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="15.5">
-      <c r="A1" s="2" t="s">
-        <v>22</v>
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>form_title</t>
+        </is>
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
@@ -1272,7 +1293,7 @@
       </c>
       <c r="C2" s="4" t="str">
         <f>TEXT(NOW(),"yyyy-mm-dd_HH-MM")</f>
-        <v>2019-04-16 12-35</v>
+        <v>2019-05-06 16-41</v>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Adjusting age validation to remove explicit question of if people are under 5
</commit_message>
<xml_diff>
--- a/forms/contact/person-create.xlsx
+++ b/forms/contact/person-create.xlsx
@@ -45,6 +45,9 @@
     <t>inputs</t>
   </si>
   <si>
+    <t>NO_LABEL</t>
+  </si>
+  <si>
     <t>user</t>
   </si>
   <si>
@@ -82,9 +85,6 @@
   </si>
   <si>
     <t>sex</t>
-  </si>
-  <si>
-    <t>select_one yes_no</t>
   </si>
   <si>
     <t>meta</t>
@@ -189,7 +189,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:Q51"/>
+  <dimension ref="A1:Q49"/>
   <sheetFormatPr defaultRowHeight="13"/>
   <cols>
     <col min="1" max="1" style="0" width="26.863281249999996" bestFit="1" customWidth="1"/>
@@ -297,6 +297,9 @@
       <c r="B2" t="s">
         <v>5</v>
       </c>
+      <c r="C2" t="s">
+        <v>6</v>
+      </c>
       <c r="F2" t="b">
         <v>0</v>
       </c>
@@ -306,15 +309,18 @@
         <v>4</v>
       </c>
       <c r="B3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="4" spans="1:17" customHeight="1" ht="13.5">
       <c r="A4" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B4" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -324,10 +330,10 @@
     </row>
     <row r="5" spans="1:17" customHeight="1" ht="13.5">
       <c r="A5" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B5" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -337,7 +343,7 @@
     </row>
     <row r="6" spans="1:17" customHeight="1" ht="13.5">
       <c r="A6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B6" t="s">
         <v>1</v>
@@ -350,35 +356,41 @@
     </row>
     <row r="7" spans="1:17" customHeight="1" ht="13.5">
       <c r="A7" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
           <t>district</t>
         </is>
+      </c>
+      <c r="C7" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="8" spans="1:17" customHeight="1" ht="13.5">
       <c r="A8" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
           <t>shehia</t>
         </is>
+      </c>
+      <c r="C8" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="9" spans="1:17" customHeight="1" ht="13.5">
       <c r="A9" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B9" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10" spans="1:17" customHeight="1" ht="13.5">
       <c r="A10" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B10" t="s">
         <v>5</v>
@@ -386,13 +398,13 @@
     </row>
     <row r="11" spans="1:17" customHeight="1" ht="13.5">
       <c r="A11" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B11" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G11" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="L11" t="inlineStr">
         <is>
@@ -402,13 +414,13 @@
     </row>
     <row r="12" spans="1:17" customHeight="1" ht="13.5">
       <c r="A12" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B12" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G12" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
@@ -418,13 +430,13 @@
     </row>
     <row r="13" spans="1:17" customHeight="1" ht="13.5">
       <c r="A13" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B13" t="s">
         <v>1</v>
       </c>
       <c r="G13" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
@@ -434,7 +446,7 @@
     </row>
     <row r="14" spans="1:17" customHeight="1" ht="13.5">
       <c r="A14" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -449,7 +461,7 @@
     </row>
     <row r="15" spans="1:17" customHeight="1" ht="13.5">
       <c r="A15" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -467,7 +479,7 @@
         <v>4</v>
       </c>
       <c r="B16" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -487,7 +499,7 @@
     </row>
     <row r="17" spans="1:17" ht="13.5">
       <c r="A17" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -507,29 +519,35 @@
     </row>
     <row r="18" spans="1:17" ht="13.5">
       <c r="A18" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B18" t="s">
         <v>0</v>
       </c>
+      <c r="C18" t="s">
+        <v>6</v>
+      </c>
       <c r="G18" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="P18" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="19" spans="1:17" ht="13.5">
       <c r="A19" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
           <t>parent</t>
         </is>
       </c>
+      <c r="C19" t="s">
+        <v>6</v>
+      </c>
       <c r="G19" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="L19" t="inlineStr">
         <is>
@@ -544,7 +562,7 @@
     </row>
     <row r="20" spans="1:17" ht="13.5">
       <c r="A20" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -562,10 +580,10 @@
         </is>
       </c>
       <c r="E20" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="I20" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J20" t="inlineStr">
         <is>
@@ -575,7 +593,7 @@
     </row>
     <row r="21" spans="1:17" ht="13.5">
       <c r="A21" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -593,10 +611,10 @@
         </is>
       </c>
       <c r="E21" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="I21" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J21" t="inlineStr">
         <is>
@@ -606,7 +624,7 @@
     </row>
     <row r="22" spans="1:17" ht="13.5">
       <c r="A22" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -621,7 +639,7 @@
     </row>
     <row r="23" spans="1:17" ht="13.5">
       <c r="A23" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -636,7 +654,7 @@
     </row>
     <row r="24" spans="1:17" ht="13.5">
       <c r="A24" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B24" t="s">
         <v>1</v>
@@ -654,7 +672,7 @@
         </is>
       </c>
       <c r="B25" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -667,12 +685,12 @@
         </is>
       </c>
       <c r="E25" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="26" spans="1:17" ht="13.5">
       <c r="A26" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -686,8 +704,10 @@
       </c>
     </row>
     <row r="27" spans="1:17" ht="13.5">
-      <c r="A27" t="s">
-        <v>19</v>
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>select_one yes_no</t>
+        </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -705,12 +725,12 @@
         </is>
       </c>
       <c r="E27" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="28" spans="1:17" ht="13.5">
       <c r="A28" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -724,325 +744,295 @@
       </c>
     </row>
     <row r="29" spans="1:17" ht="13.5">
-      <c r="A29" t="s">
-        <v>19</v>
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>is_under_5</t>
+          <t>yob</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>ASK: Is ${first_name_c} under 5 years old?</t>
+          <t>ASK: In what year was ${first_name_c} born?</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>ULIZA: Je mtoto yupo chini ya umri wa miaka 5?</t>
+          <t>ULIZA: Ni mwaka gani alizaliwa?</t>
         </is>
       </c>
       <c r="E29" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>selected(${exact_dob_known_c},"no")</t>
+          <t>${exact_dob_known_c}="no"</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>format-date-time(today(),"%Y") - . &gt; 5 and format-date-time(today(),"%Y") - . &lt;= 100</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>For children under 5 years of age, a more exact birthdate must be captured. Please select "Yes" to the prior question and do your best to capture a more exact birthdate.</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>Kwa watoto walio chini ya umri wa miaka 5, tarehe yake yao ya kuzaliwa nilazima ichukuliwe.</t>
         </is>
       </c>
     </row>
     <row r="30" spans="1:17" ht="13.5">
-      <c r="A30" t="s">
-        <v>14</v>
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>under_5_dob_note</t>
+          <t>dob</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>SAY: For children under 5, I'd like to try and get some more specific information about their age. Can you try and remember the year and month when ${first_name_c} was born?</t>
+          <t>ASK: What is ${first_name_c}'s date of birth?</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>SEMA: Kwa watoto walio chini ya miaka 5 ningependa kupata taarifa zaidi kuhusu umri wao. Je,, unaweza kukumbuka ni mwezi na mwaka gani mtoto huyu alizaliwa?</t>
-        </is>
+          <t>ULIZA: Ipi ni tarehe yake kuzaliwa</t>
+        </is>
+      </c>
+      <c r="E30" t="s">
+        <v>17</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>selected(${exact_dob_known_c},"no") and selected(${is_under_5},"yes")</t>
-        </is>
-      </c>
-      <c r="N30" t="inlineStr">
-        <is>
-          <t>It's important to try and get more exact age information for children. You can enter the child's date of birth as the first of the month in which they were born.</t>
-        </is>
-      </c>
-      <c r="O30" t="inlineStr">
-        <is>
-          <t>Ni muhimu kupata taarifa za uhakika kuhuru umri wa watoto. Unaweza kuingiza tarehe ya mwezi wa mtoto aliozaliwa</t>
+          <t>${exact_dob_known_c}="yes"</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>. &lt;= date-time(decimal-date-time(today())) and . &gt;= date-time(decimal-date-time(today() - (100 * 365.25)))</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>You've entered a birthdate either in the future or very long ago - confirm that you've entered it properly.</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>Je umeingiza umri sahihi- hakikisha umeingiza kwa usahihi. Kwa watoto walio chini ya miaka 5, hakikisha kuwa tarehe yao si ya Zaidi ya miaka 5 nyuma.</t>
         </is>
       </c>
     </row>
     <row r="31" spans="1:17" ht="13.5">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>integer</t>
-        </is>
+      <c r="A31" t="s">
+        <v>12</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>yob</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>ASK: In what year was ${first_name_c} born?</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>ULIZA: Ni mwaka gani alizaliwa?</t>
-        </is>
-      </c>
-      <c r="E31" t="s">
-        <v>16</v>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>selected(${exact_dob_known_c},"no") and selected(${is_under_5},"no")</t>
-        </is>
-      </c>
-      <c r="I31" t="inlineStr">
-        <is>
-          <t>format-date-time(today(),"%Y") - . &gt; 5 and format-date-time(today(),"%Y") - . &lt;= 100</t>
-        </is>
-      </c>
-      <c r="J31" t="inlineStr">
-        <is>
-          <t>For children under 5 years of age, a more exact birthdate must be captured.</t>
-        </is>
-      </c>
-      <c r="K31" t="inlineStr">
-        <is>
-          <t>Kwa watoto walio chini ya umri wa miaka 5, tarehe yake yao ya kuzaliwa nilazima ichukuliwe.</t>
+          <t>date_of_birth</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>format-date(if(../dob != '', ../dob,concat(../yob, '-01-01')), '%Y-%m-%d')</t>
         </is>
       </c>
     </row>
     <row r="32" spans="1:17" ht="13.5">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>date</t>
-        </is>
+      <c r="A32" t="s">
+        <v>12</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>dob</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>ASK: What is ${first_name_c}'s date of birth?</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>ULIZA: Ipi ni tarehe yake kuzaliwa</t>
-        </is>
-      </c>
-      <c r="E32" t="s">
-        <v>16</v>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>selected(${exact_dob_known_c},"yes") or (selected(${exact_dob_known_c},"no") and selected(${is_under_5},"yes"))</t>
-        </is>
-      </c>
-      <c r="I32" t="inlineStr">
-        <is>
-          <t>(selected(${is_under_5},"yes") and . &lt;= date-time(decimal-date-time(today())) and . &gt; date-time(decimal-date-time(today() - (5 * 365.25)))) or (${exact_dob_known_c}="yes" and . &lt;= date-time(decimal-date-time(today())) and . &gt;= date-time(decimal-date-time(today() - (100 * 365.25))))</t>
-        </is>
-      </c>
-      <c r="J32" t="inlineStr">
-        <is>
-          <t>You've entered an invalid age - confirm that you've entered it properly.  For children under 5, confirm that the date is not more than 5 years ago.</t>
-        </is>
-      </c>
-      <c r="K32" t="inlineStr">
-        <is>
-          <t>Je umeingiza umri sahihi- hakikisha umeingiza kwa usahihi. Kwa watoto walio chini ya miaka 5, hakikisha kuwa tarehe yao si ya Zaidi ya miaka 5 nyuma.</t>
+          <t>date_of_birth_c</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>../date_of_birth</t>
         </is>
       </c>
     </row>
     <row r="33" spans="1:17" ht="13.5">
       <c r="A33" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>date_of_birth</t>
+          <t>reproductive_age</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>format-date(if(../dob != '', ../dob,concat(../yob, '-01-01')), '%Y-%m-%d')</t>
+          <t>if(${sex_c}="female" and ((((decimal-date-time(today()) - decimal-date-time(${date_of_birth_c})) div 365) &gt;= 15 and ((decimal-date-time(today()) - decimal-date-time(${date_of_birth_c})) div 365) &lt;= 49)),int(1),int(0))</t>
         </is>
       </c>
     </row>
     <row r="34" spans="1:17" ht="13.5">
       <c r="A34" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>date_of_birth_c</t>
+          <t>is_under_5_binary</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>../date_of_birth</t>
+          <t>if(${exact_dob_known_c}="yes",if(((decimal-date-time(today()) - decimal-date-time(${date_of_birth_c})) div 365.25) &lt; 5,1,0),0)</t>
         </is>
       </c>
     </row>
     <row r="35" spans="1:17" ht="13.5">
       <c r="A35" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>reproductive_age</t>
-        </is>
-      </c>
-      <c r="L35" t="inlineStr">
-        <is>
-          <t>if(${sex_c}="female" and ((((decimal-date-time(today()) - decimal-date-time(${date_of_birth_c})) div 365) &gt;= 15 and ((decimal-date-time(today()) - decimal-date-time(${date_of_birth_c})) div 365) &lt;= 49)),int(1),int(0))</t>
+          <t>return_children_note</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>SAY: From this registration, I've seen that you have a child under 5 who can benefit from this national program. Therefore, I'm asking for your permission to come back and check up on all issues related to their health care, nutrition, and child development. I would be grateful for your permission.</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>SEMA kutokanana usajili huu nimeona kuna watoto walio chini ya umri wa miaka 5 ambao wanaweza kunufaika na mradi huu wa kitaifa. Kwahivyo naomba ridhaa ya kurudi tena ili nije kuangalia maswala yote yanayohusiana na huduma zao za afya, lishe, na maendeleo yao. Nitafurahi kama nitapata ridhaa yenu.</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>${is_under_5_binary}=1</t>
         </is>
       </c>
     </row>
     <row r="36" spans="1:17" ht="13.5">
       <c r="A36" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>is_under_5_binary</t>
-        </is>
-      </c>
-      <c r="L36" t="inlineStr">
-        <is>
-          <t>if(selected(${exact_dob_known_c},"yes"),if(((decimal-date-time(today()) - decimal-date-time(${date_of_birth_c})) div 365.25) &lt; 5,1,0),if(selected(${is_under_5},"yes"),int(1),int(0)))</t>
-        </is>
+          <t>return_women_note</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>SAY: I see that there are some women of reproductive age in your family. I'd like to ask your permission to return later to speak with them personally about issues related to health during pregnancy and childbirth.</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>SEMA: Nimeona kuna baadhi ya wanawake walio katika umri wa uzazi katika kaya yako. Ningeomba ridhaa yako kurudia ili kuja kuzungumza nao mambo muhimu ya afya kipindi cha ujauzito na baada ya kujifungua.</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>${reproductive_age} = 1</t>
+        </is>
+      </c>
+      <c r="G36" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="37" spans="1:17" ht="13.5">
       <c r="A37" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>return_children_note</t>
+          <t>debug_note</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>SAY: From this registration, I've seen that you have a child under 5 who can benefit from this national program. Therefore, I'm asking for your permission to come back and check up on all issues related to their health care, nutrition, and child development. I would be grateful for your permission.</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>SEMA kutokanana usajili huu nimeona kuna watoto walio chini ya umri wa miaka 5 ambao wanaweza kunufaika na mradi huu wa kitaifa. Kwahivyo naomba ridhaa ya kurudi tena ili nije kuangalia maswala yote yanayohusiana na huduma zao za afya, lishe, na maendeleo yao. Nitafurahi kama nitapata ridhaa yenu.</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>${is_under_5_binary}=1</t>
-        </is>
+          <t>date of birth: ${date_of_birth_c} under_5_flag: ${is_under_5_binary} is reproductive age: ${reproductive_age}</t>
+        </is>
+      </c>
+      <c r="G37" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="38" spans="1:17" ht="13.5">
       <c r="A38" t="s">
-        <v>14</v>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>return_women_note</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>SAY: I see that there are some women of reproductive age in your family. I'd like to ask your permission to return later to speak with them personally about issues related to health during pregnancy and childbirth.</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>SEMA: Nimeona kuna baadhi ya wanawake walio katika umri wa uzazi katika kaya yako. Ningeomba ridhaa yako kurudia ili kuja kuzungumza nao mambo muhimu ya afya kipindi cha ujauzito na baada ya kujifungua.</t>
-        </is>
-      </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>${reproductive_age} = 1</t>
-        </is>
-      </c>
-      <c r="G38" t="s">
-        <v>12</v>
+        <v>4</v>
+      </c>
+      <c r="B38" t="s">
+        <v>20</v>
+      </c>
+      <c r="C38" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="39" spans="1:17" ht="13.5">
       <c r="A39" t="s">
-        <v>14</v>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>debug_note</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>date of birth: ${date_of_birth_c} under_5_flag: ${is_under_5_binary} is reproductive age: ${reproductive_age}</t>
-        </is>
-      </c>
-      <c r="G39" t="s">
-        <v>12</v>
+        <v>21</v>
+      </c>
+      <c r="B39" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="40" spans="1:17" ht="13.5">
       <c r="A40" t="s">
-        <v>4</v>
+        <v>22</v>
       </c>
       <c r="B40" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="41" spans="1:17" ht="13.5">
       <c r="A41" t="s">
-        <v>21</v>
-      </c>
-      <c r="B41" t="s">
-        <v>21</v>
+        <v>12</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>created_by</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>../../../name</t>
+        </is>
       </c>
     </row>
     <row r="42" spans="1:17" ht="13.5">
       <c r="A42" t="s">
-        <v>22</v>
-      </c>
-      <c r="B42" t="s">
-        <v>22</v>
+        <v>12</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>created_by_person_uuid</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>../../../contact_id</t>
+        </is>
       </c>
     </row>
     <row r="43" spans="1:17" ht="13.5">
       <c r="A43" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>created_by</t>
+          <t>created_by_place_uuid</t>
         </is>
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>../../../name</t>
+          <t>../../../facility_id</t>
         </is>
       </c>
     </row>
@@ -1050,53 +1040,23 @@
       <c r="A44" t="s">
         <v>11</v>
       </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>created_by_person_uuid</t>
-        </is>
-      </c>
-      <c r="L44" t="inlineStr">
-        <is>
-          <t>../../../contact_id</t>
-        </is>
+      <c r="B44" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="45" spans="1:17" ht="13.5">
       <c r="A45" t="s">
         <v>11</v>
       </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>created_by_place_uuid</t>
-        </is>
-      </c>
-      <c r="L45" t="inlineStr">
-        <is>
-          <t>../../../facility_id</t>
-        </is>
-      </c>
-    </row>
-    <row r="46" spans="1:17" ht="13.5">
-      <c r="A46" t="s">
-        <v>10</v>
-      </c>
-      <c r="B46" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="47" spans="1:17" ht="13.5">
-      <c r="A47" t="s">
-        <v>10</v>
-      </c>
-      <c r="B47" t="s">
-        <v>13</v>
-      </c>
+      <c r="B45" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="47" spans="1:17">
+      <c r="D47" s="1"/>
     </row>
     <row r="49" spans="1:17">
       <c r="D49" s="1"/>
-    </row>
-    <row r="51" spans="1:17">
-      <c r="D51" s="1"/>
     </row>
   </sheetData>
   <sheetProtection formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" selectLockedCells="1" sort="0" autoFilter="0" pivotTables="0" selectUnlockedCells="1"/>
@@ -1146,7 +1106,7 @@
         <v>23</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
@@ -1181,7 +1141,7 @@
     </row>
     <row r="4" spans="1:4" ht="14.75">
       <c r="A4" s="3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
@@ -1201,7 +1161,7 @@
     </row>
     <row r="5" spans="1:4" ht="14.75">
       <c r="A5" s="3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
@@ -1293,7 +1253,7 @@
       </c>
       <c r="C2" s="4" t="str">
         <f>TEXT(NOW(),"yyyy-mm-dd_HH-MM")</f>
-        <v>2019-05-06 16-41</v>
+        <v>2019-05-07 10-28</v>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>

</xml_diff>